<commit_message>
feat: Term of the Week 2026-W41 (Fashiontainment), AI Slop entry, linked related terms
- W41 pick: Fashiontainment (Gap Inc. x JYT, 22 Sep 2026), fact-checked
- New regular entry: AI Slop, cross-linked to Workslop
- Related terms now link to matching public entries (term pages and dialog)
- Backup backup-2026-10-05-tow/, report reports/term-of-week-2026-W41.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source/MMA_Dictionary_Master_Glossary_v1.xlsx
+++ b/source/MMA_Dictionary_Master_Glossary_v1.xlsx
@@ -170,7 +170,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MMADictionaryGlossary" displayName="MMADictionaryGlossary" ref="A1:T370" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MMADictionaryGlossary" displayName="MMADictionaryGlossary" ref="A1:T372" headerRowCount="1">
   <autoFilter ref="A1:Q103"/>
   <tableColumns count="20">
     <tableColumn id="1" name="Term"/>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T370"/>
+  <dimension ref="A1:T372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -18398,12 +18398,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Humanwashing</t>
+          <t>AI Slop</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -18413,32 +18413,32 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>The practice of making AI-assisted work look fully human-made, through handcrafted styling, named creators or behind-the-scenes stories, while hiding how much AI actually did.</t>
+          <t>Low-quality content made in bulk with generative AI, published to fill feeds and collect views or ad money rather than to inform or entertain.</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Humanwashing is the mirror image of AI washing: instead of overstating AI to borrow a tech halo, a brand understates AI to protect an authenticity halo. Business ethicist Peter Seele introduced 'humanwashing of machines' in a March 2021 post, and in 2022 formalized it with Andreea Scorici and Mario Schultz in AI &amp; Society as the deceptive use of a machine's human-like appearance to mislead people about what it can really do. Marketing writers then took the word over for brand and creative work: the WHAT'S ANU newsletter in December 2025, followed by agencies such as Flux+Form in 2026, where it now means passing off AI-generated content as human craft. The risk for marketers is trust: when undisclosed AI use surfaces, the brand is judged less on the AI itself than on the concealment.</t>
+          <t>AI slop is the flood of cheap AI-generated images, videos, articles and posts that now fills social feeds, video platforms and search results. It is usually made fast, at scale and with little human checking, so it tends to be repetitive, wrong or strange. The word 'slop' first meant liquid waste or scraps fed to pigs. Its use for low-grade AI output apparently began around 2022, after AI image generators were released, among commenters on 4chan, Hacker News and YouTube. British programmer Simon Willison was an early champion of the term: in a blog post on 8 May 2024 he argued for using it and credited a tweet that said 'slop' was becoming a term of art. Merriam-Webster and the American Dialect Society both named 'slop' their 2025 Word of the Year. It is a close relative of workslop: workslop is polished-looking AI output inside a company that leaves colleagues with extra work, while AI slop is published to public feeds and platforms. For advertisers the term matters in two ways: ads can run next to slop, and AI-made creative can be read as slop by audiences, so media plans need adjacency checks and creative needs a human quality bar.</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>In August 2025 J.Crew posted AI-generated images styled as vintage catalog shots on Instagram without saying they were AI-made. After the newsletter Blackbird Spyplane exposed them on 26 August 2025, the brand edited its captions to credit an 'AI photographer' rather than stating plainly that the images were AI-generated.</t>
+          <t>In November 2024, Coca-Cola released AI-generated holiday commercials that were met with backlash from viewers and artists. On 1 October 2026, Digiday reported that Pixability had launched Pixie, a tool that filters AI slop out of YouTube ad buys using a combination of human verification and AI. Pixability chief product officer Jackie Paulino said Pixie removes "MFA content, nefarious content, things that are generated really as clickbait".</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>MMA Sözlük (Term of the Week)</t>
+          <t>MMA Sözlük (Research 2026)</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>https://flux-form.com/what-is-humanwashing/ https://whatsanu.substack.com/p/2510-humanwashing https://www.blackbirdspyplane.com/p/jcrew-used-ai-to-counterfeit-their-own-vibes https://www.adweek.com/creativity/in-2026-brands-are-virtue-signaling-about-ai/ https://businessesgrow.com/2026/09/21/human-moat/ https://petapixel.com/2025/09/02/j-crews-ai-generated-fashion-images-look-a-lot-like-real-photos/ https://www.mmaglobal.com/rail</t>
+          <t>https://digiday.com/media-buying/as-ai-slop-spreads-pixability-offers-a-way-to-root-it-out-on-youtube/ https://www.adweek.com/agencies/red-antler-owned-creator-studio-wants-to-fight-ai-slop-with-ugc/ https://digiday.com/marketing/the-creator-economys-stance-on-ai-is-shifting-again/ https://en.wikipedia.org/wiki/AI_slop https://simonwillison.net/2024/May/8/slop/ https://www.americandialect.org/2025-word-of-the-year-is-slop https://en.wiktionary.org/wiki/slop</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>AI Washing, Synthetic Trust, Synthetic Influence, Responsible AI, Greenwashing</t>
+          <t>Workslop, Brain Rot, MFA (Made-for-Advertising), Humanwashing, Synthetic Trust</t>
         </is>
       </c>
       <c r="J311" t="inlineStr">
@@ -18448,39 +18448,29 @@
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>Humanwashing, yapay zeka ile üretilen bir işi el emeği görünümü, isimlendirilmiş yaratıcılar ya da kamera arkası hikâyelerle tamamen insan yapımı gibi sunarak yapay zekanın katkısını gizlemektir.</t>
+          <t>AI slop, bilgi vermek ya da eğlendirmek yerine akışları doldurup izlenme veya reklam geliri toplamak için yapay zeka ile toplu halde üretilen düşük kaliteli içeriktir.</t>
         </is>
       </c>
       <c r="N311" t="inlineStr">
         <is>
-          <t>Term of the Week 2026-W39</t>
+          <t>Draft (researched 2026-09-23)</t>
         </is>
       </c>
       <c r="Q311" t="inlineStr">
         <is>
-          <t>Recency: no source dated in the last 14 days uses the exact word; the topic is current through adjacent coverage (Schaefer, 21 Sep 2026). Seele's original sense differs from the marketing sense; both are stated. Fact-checked 2026-09-23.</t>
-        </is>
-      </c>
-      <c r="S311" t="inlineStr">
-        <is>
-          <t>The question sits in the territory of MMA's AI Leadership Think Tank (ALTT, formerly the AI Leadership Coalition), which runs a Responsible AI working group and the Responsible AI Innovation Lab (RAIL), a source of guidelines, templates and checklists for ethical AI use in marketing. It is also the counterpart of AI Washing, already in this dictionary: one overclaims AI, the other hides it, and both erode the same asset, consumer trust.</t>
-        </is>
-      </c>
-      <c r="T311" t="inlineStr">
-        <is>
-          <t>2026-W39 | As the 2026 backlash against AI-made ads grows, brands are tempted to hide their AI use behind handmade, human-looking work. This week's coverage of the 'human moat' as the last brand differentiator puts that trade-off on the table.</t>
+          <t>No single coiner; the 2022 early use is reported by Wikipedia as approximate, and Willison (May 2024) popularized the term rather than coined it. Merriam-Webster's Word of the Year page could not be opened (403); the pick is confirmed via the American Dialect Society page and Wikipedia. Adweek article dated only October 2026. Fact-checked 2026-10-05. Considered for Term of the Week 2026-W41 and added as a regular entry instead.</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Frankenstack</t>
+          <t>Humanwashing</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>H</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -18490,17 +18480,17 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>A marketing or advertising technology stack assembled from many separately bought tools that were bolted together over time and do not work as one system.</t>
+          <t>The practice of making AI-assisted work look fully human-made, through handcrafted styling, named creators or behind-the-scenes stories, while hiding how much AI actually did.</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>A Frankenstack is what a marketing team ends up with when each department buys its own tools for data, media buying, creative and reporting, and the pieces are later wired together with manual work, exports and custom connectors. The word blends Frankenstein and tech stack: a system built from mismatched parts that runs, but badly. It comes from the martech world. The earliest verifiable use found is a 31 March 2015 chiefmartec.com post by its editor Scott Brinker, who wrote that the phrase had entered the industry's lingo; six weeks later, in a CIO.com interview, he called it a 'humorous label' for stacks that grew out of marketing silos. No single coiner is known. In 2025 and 2026 the term returned in adtech coverage as teams started adding AI tools and agents on top of these stacks. Before a team adds another AI tool, it pays to check whether the tool connects the existing data and workflows or just adds one more part to the stack.</t>
+          <t>Humanwashing is the mirror image of AI washing: instead of overstating AI to borrow a tech halo, a brand understates AI to protect an authenticity halo. Business ethicist Peter Seele introduced 'humanwashing of machines' in a March 2021 post, and in 2022 formalized it with Andreea Scorici and Mario Schultz in AI &amp; Society as the deceptive use of a machine's human-like appearance to mislead people about what it can really do. Marketing writers then took the word over for brand and creative work: the WHAT'S ANU newsletter in December 2025, followed by agencies such as Flux+Form in 2026, where it now means passing off AI-generated content as human craft. The risk for marketers is trust: when undisclosed AI use surfaces, the brand is judged less on the AI itself than on the concealment.</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>In the 8 September 2026 episode of MMA's Decoding AI for Marketing podcast, hosted by Greg Stuart and Rex Briggs, Fluency CEO Mike Lane described advertising execution as still largely manual. The episode notes say that when fragmented platforms are stitched together with new AI tools, they can create what Lane calls a 'Frankenstack' of software, and that he argues for integrated operating systems that connect data, media and AI agents. At Advertising Week 2025, adtech company Infillion framed the trend as 'the end of the Frankenstack' and a move to composable ad tech (Infillion blog, 9 October 2025).</t>
+          <t>In August 2025 J.Crew posted AI-generated images styled as vintage catalog shots on Instagram without saying they were AI-made. After the newsletter Blackbird Spyplane exposed them on 26 August 2025, the brand edited its captions to credit an 'AI photographer' rather than stating plainly that the images were AI-generated.</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -18510,54 +18500,54 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>https://www.decodingaiformarketing.com/ https://podcasts.apple.com/us/podcast/decoding-ai-for-marketing/id1715735755 https://chiefmartec.com/2015/03/springtime-marketing-technology-martech/ https://www.cio.com/article/246971/marketing-tech-prosfrankenstack-tools-and-the-future.html https://infillion.com/blog/advertising-week-2025-the-end-of-the-frankenstack-and-the-rise-of-composable-ad-tech/</t>
+          <t>https://flux-form.com/what-is-humanwashing/ https://whatsanu.substack.com/p/2510-humanwashing https://www.blackbirdspyplane.com/p/jcrew-used-ai-to-counterfeit-their-own-vibes https://www.adweek.com/creativity/in-2026-brands-are-virtue-signaling-about-ai/ https://businessesgrow.com/2026/09/21/human-moat/ https://petapixel.com/2025/09/02/j-crews-ai-generated-fashion-images-look-a-lot-like-real-photos/ https://www.mmaglobal.com/rail</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
         <is>
-          <t>Workflow-First AI, AI Wrapper, AI Orchestrator, CDP / Customer Data Platform, MCP (Model Context Protocol)</t>
+          <t>AI Washing, Synthetic Trust, Synthetic Influence, Responsible AI, Greenwashing</t>
         </is>
       </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>Technology Trends</t>
+          <t>AI &amp; Marketing Concepts</t>
         </is>
       </c>
       <c r="L312" t="inlineStr">
         <is>
-          <t>Frankenstack, zamanla ayrı ayrı alınıp birbirine eklenen ve tek bir sistem gibi çalışmayan araçlardan oluşan pazarlama ya da reklam teknolojisi altyapısıdır.</t>
+          <t>Humanwashing, yapay zeka ile üretilen bir işi el emeği görünümü, isimlendirilmiş yaratıcılar ya da kamera arkası hikâyelerle tamamen insan yapımı gibi sunarak yapay zekanın katkısını gizlemektir.</t>
         </is>
       </c>
       <c r="N312" t="inlineStr">
         <is>
-          <t>Term of the Week 2026-W40</t>
+          <t>Term of the Week 2026-W39</t>
         </is>
       </c>
       <c r="Q312" t="inlineStr">
         <is>
-          <t>No public transcript of the episode; Mike Lane's wording is attributed through the episode notes, not quoted directly. March 2015 is the earliest verifiable use, not a proven coinage date. MMA names checked against mma-org-context. Fact-checked 2026-09-28.</t>
+          <t>Recency: no source dated in the last 14 days uses the exact word; the topic is current through adjacent coverage (Schaefer, 21 Sep 2026). Seele's original sense differs from the marketing sense; both are stated. Fact-checked 2026-09-23.</t>
         </is>
       </c>
       <c r="S312" t="inlineStr">
         <is>
-          <t>The term was the subject of an episode of MMA's own Decoding AI for Marketing podcast, hosted by MMA CEO Greg Stuart and Rex Briggs. The topic sits in the territory of MMA's AI Leadership Think Tank (ALTT), whose working groups include Audience Dev &amp; Media Buying, and of the AI/Org Transformation priority on MMA's 2026 agenda, which covers operating models for AI. MMA's State of Agentic AI in Marketing (2026) report is the related reading for teams planning to add AI agents to an existing stack.</t>
+          <t>The question sits in the territory of MMA's AI Leadership Think Tank (ALTT, formerly the AI Leadership Coalition), which runs a Responsible AI working group and the Responsible AI Innovation Lab (RAIL), a source of guidelines, templates and checklists for ethical AI use in marketing. It is also the counterpart of AI Washing, already in this dictionary: one overclaims AI, the other hides it, and both erode the same asset, consumer trust.</t>
         </is>
       </c>
       <c r="T312" t="inlineStr">
         <is>
-          <t>2026-W40 | On 8 September 2026, MMA's Decoding AI for Marketing podcast asked whether AI can fix advertising's Frankenstack. Guest Mike Lane, CEO of Fluency, argued that stitching new AI tools onto fragmented platforms can create one instead.</t>
+          <t>2026-W39 | As the 2026 backlash against AI-made ads grows, brands are tempted to hide their AI use behind handmade, human-looking work. This week's coverage of the 'human moat' as the last brand differentiator puts that trade-off on the table.</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>MOSTT (Marketing Organization Structure Think Tank)</t>
+          <t>Frankenstack</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -18567,44 +18557,74 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>A think tank focused on analyzing and optimizing marketing organization structures.</t>
+          <t>A marketing or advertising technology stack assembled from many separately bought tools that were bolted together over time and do not work as one system.</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>A Frankenstack is what a marketing team ends up with when each department buys its own tools for data, media buying, creative and reporting, and the pieces are later wired together with manual work, exports and custom connectors. The word blends Frankenstein and tech stack: a system built from mismatched parts that runs, but badly. It comes from the martech world. The earliest verifiable use found is a 31 March 2015 chiefmartec.com post by its editor Scott Brinker, who wrote that the phrase had entered the industry's lingo; six weeks later, in a CIO.com interview, he called it a 'humorous label' for stacks that grew out of marketing silos. No single coiner is known. In 2025 and 2026 the term returned in adtech coverage as teams started adding AI tools and agents on top of these stacks. Before a team adds another AI tool, it pays to check whether the tool connects the existing data and workflows or just adds one more part to the stack.</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>In the 8 September 2026 episode of MMA's Decoding AI for Marketing podcast, hosted by Greg Stuart and Rex Briggs, Fluency CEO Mike Lane described advertising execution as still largely manual. The episode notes say that when fragmented platforms are stitched together with new AI tools, they can create what Lane calls a 'Frankenstack' of software, and that he argues for integrated operating systems that connect data, media and AI agents. At Advertising Week 2025, adtech company Infillion framed the trend as 'the end of the Frankenstack' and a move to composable ad tech (Infillion blog, 9 October 2025).</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>MMA Sözlük / MMA Acronyms.docx</t>
+          <t>MMA Sözlük (Term of the Week)</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://www.decodingaiformarketing.com/ https://podcasts.apple.com/us/podcast/decoding-ai-for-marketing/id1715735755 https://chiefmartec.com/2015/03/springtime-marketing-technology-martech/ https://www.cio.com/article/246971/marketing-tech-prosfrankenstack-tools-and-the-future.html https://infillion.com/blog/advertising-week-2025-the-end-of-the-frankenstack-and-the-rise-of-composable-ad-tech/</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Workflow-First AI, AI Wrapper, AI Orchestrator, CDP / Customer Data Platform, MCP (Model Context Protocol)</t>
         </is>
       </c>
       <c r="J313" t="inlineStr">
         <is>
-          <t>MMA Programs &amp; Frameworks</t>
-        </is>
-      </c>
-      <c r="K313" t="inlineStr">
-        <is>
-          <t>Pazarlama Organizasyon Yapısı Düşünce Grubu</t>
+          <t>Technology Trends</t>
         </is>
       </c>
       <c r="L313" t="inlineStr">
         <is>
-          <t>Pazarlama organizasyon yapılarını analiz eden ve optimize eden düşünce grubudur.</t>
+          <t>Frankenstack, zamanla ayrı ayrı alınıp birbirine eklenen ve tek bir sistem gibi çalışmayan araçlardan oluşan pazarlama ya da reklam teknolojisi altyapısıdır.</t>
         </is>
       </c>
       <c r="N313" t="inlineStr">
         <is>
-          <t>Source list</t>
+          <t>Term of the Week 2026-W40</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>No public transcript of the episode; Mike Lane's wording is attributed through the episode notes, not quoted directly. March 2015 is the earliest verifiable use, not a proven coinage date. MMA names checked against mma-org-context. Fact-checked 2026-09-28.</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>The term was the subject of an episode of MMA's own Decoding AI for Marketing podcast, hosted by MMA CEO Greg Stuart and Rex Briggs. The topic sits in the territory of MMA's AI Leadership Think Tank (ALTT), whose working groups include Audience Dev &amp; Media Buying, and of the AI/Org Transformation priority on MMA's 2026 agenda, which covers operating models for AI. MMA's State of Agentic AI in Marketing (2026) report is the related reading for teams planning to add AI agents to an existing stack.</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>2026-W40 | On 8 September 2026, MMA's Decoding AI for Marketing podcast asked whether AI can fix advertising's Frankenstack. Guest Mike Lane, CEO of Fluency, argued that stitching new AI tools onto fragmented platforms can create one instead.</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MARS (Mobile, Analytics, Real-Time, Social)</t>
+          <t>Fashiontainment</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -18614,39 +18634,69 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>A framework for marketing strategies that integrate mobile, analytics, real-time decision-making, and social media.</t>
+          <t>A brand strategy in which a fashion company acts like an entertainment business, building fandom through content, music, live experiences and licensing instead of relying on ad campaigns alone.</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Fashiontainment treats a clothing brand as a source of stories and cultural moments, not only of products. The brand co-produces shows, partners with artists, runs live events and designs collections with the talent, so fans meet it inside the entertainment they already follow. The word blends fashion and entertainment. Gap Inc. CEO Richard Dickson uses the word to describe the company's strategy. In January 2026 Gap Inc. announced the hire of former Paramount executive Pam Kaufman (starting 2 February) in the newly created role of Chief Entertainment Officer; Retail Dive reported his view that 'fashion is entertainment', or 'fashiontainment'. Gap Inc. now uses Fashiontainment as the name of the platform Kaufman leads. Like edutainment and archivetainment, it is built by joining a field's name with 'entertainment'. For marketers, the test is whether a partnership builds a lasting fan relationship across content, stores and product, or is simply a celebrity campaign with a new name.</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>On 22 September 2026, Gap Inc. announced a multi-year partnership with Just Your Type (JYT), a five-member boy band developed by songwriter and producer Freddy Wexler and signed to Wexler Records and Republic Records. It is the first collaboration under Gap Inc.'s Fashiontainment platform. The plan includes a multi-episode docuseries co-produced by Gap, a national mall tour, a Gap capsule collection co-designed with the band's five members and social content. Gap Inc. said JYT had generated more than 450 million views over the previous 90 days.</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>MMA Sözlük / MMA Acronyms.docx</t>
+          <t>MMA Sözlük (Term of the Week)</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://s204.q4cdn.com/320226404/files/doc_news/Gap-Inc--Debuts-First-Fashiontainment-Partnership-with-Emerging-Boy-Band-JYT-2026.pdf https://marketingdive.com/news/gap-rolls-out-fashiontainment-strategy-with-boy-band-collaboration/830984 https://www.retaildive.com/news/gap-inc-paramount-hollywood-exec-fashiontainment-role/809849/</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Archivetainment, Edutainment, Funvertising, BaP (Brand as Performance)</t>
         </is>
       </c>
       <c r="J314" t="inlineStr">
         <is>
-          <t>MMA Programs &amp; Frameworks</t>
-        </is>
-      </c>
-      <c r="K314" t="inlineStr">
-        <is>
-          <t>Mobil, Analitik, Gerçek Zamanlı, Sosyal</t>
+          <t>Consumer &amp; Culture Trends</t>
         </is>
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>Mobil ve sosyal medya pazarlaması için veri odaklı analiz yöntemleri sunar.</t>
+          <t>Fashiontainment, bir moda markasının yalnızca reklam kampanyalarına dayanmak yerine içerik, müzik, canlı deneyim ve lisanslama ile hayran kitlesi oluşturarak bir eğlence şirketi gibi çalıştığı marka stratejisidir.</t>
         </is>
       </c>
       <c r="N314" t="inlineStr">
         <is>
-          <t>Source list</t>
+          <t>Term of the Week 2026-W41</t>
+        </is>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>Retail Dive presents fashiontainment as Dickson's framing but does not say he coined the word; searches found no earlier use, and coverage from January 2026 on credits Gap Inc. The 450 million views figure is Gap Inc.'s own claim in its press release. Fact-checked 2026-10-05.</t>
+        </is>
+      </c>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>The Marketing + Media Alliance (MMA) has no published study on fashiontainment. For teams that need to show what entertainment-led brand building returns, the closest MMA work is Brand as Performance (BaP), the Marketing Attribution Think Tank (MATT) program on how brand investment converts to sales, and Brand Value, one of MMA's 2026 priorities.</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>2026-W41 | On 22 September 2026, Gap Inc. announced its first Fashiontainment partnership: a multi-year deal with the boy band JYT that includes a docuseries co-produced by Gap, a national mall tour and a capsule collection co-designed with the band.</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>MRA (MarCaps Readiness Assessment)</t>
+          <t>MOSTT (Marketing Organization Structure Think Tank)</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -18661,7 +18711,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>A diagnostic tool that evaluates an organization’s marketing capabilities and their alignment with business strategy.</t>
+          <t>A think tank focused on analyzing and optimizing marketing organization structures.</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -18676,12 +18726,12 @@
       </c>
       <c r="K315" t="inlineStr">
         <is>
-          <t>MarCaps Hazırlık Değerlendirmesi</t>
+          <t>Pazarlama Organizasyon Yapısı Düşünce Grubu</t>
         </is>
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>Pazarlama stratejilerinin ne kadar etkili olduğunu ölçen bir değerlendirme aracı.</t>
+          <t>Pazarlama organizasyon yapılarını analiz eden ve optimize eden düşünce grubudur.</t>
         </is>
       </c>
       <c r="N315" t="inlineStr">
@@ -18693,7 +18743,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>MCB (Marketing Capabilities Benchmark)</t>
+          <t>MARS (Mobile, Analytics, Real-Time, Social)</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -18708,7 +18758,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>An assessment system that measures individual team members’ marketing capabilities.</t>
+          <t>A framework for marketing strategies that integrate mobile, analytics, real-time decision-making, and social media.</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -18723,12 +18773,12 @@
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t>Pazarlama Yetkinlik Kıyaslaması</t>
+          <t>Mobil, Analitik, Gerçek Zamanlı, Sosyal</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>Pazarlama ekiplerinin yetkinlik düzeylerini belirlemek için kullanılan analiz metodu.</t>
+          <t>Mobil ve sosyal medya pazarlaması için veri odaklı analiz yöntemleri sunar.</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
@@ -18740,7 +18790,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>MATT (Marketing Attribution Think Tank)</t>
+          <t>MRA (MarCaps Readiness Assessment)</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -18755,7 +18805,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>A think tank dedicated to improving marketing attribution and proving marketing’s impact on business growth.</t>
+          <t>A diagnostic tool that evaluates an organization’s marketing capabilities and their alignment with business strategy.</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
@@ -18770,12 +18820,12 @@
       </c>
       <c r="K317" t="inlineStr">
         <is>
-          <t>Pazarlama Atıf Düşünce Grubu</t>
+          <t>MarCaps Hazırlık Değerlendirmesi</t>
         </is>
       </c>
       <c r="L317" t="inlineStr">
         <is>
-          <t>Pazarlama yatırım getirisi (ROI) ve pazarlama performansı ölçümleme konularında çalışan düşünce grubudur.</t>
+          <t>Pazarlama stratejilerinin ne kadar etkili olduğunu ölçen bir değerlendirme aracı.</t>
         </is>
       </c>
       <c r="N317" t="inlineStr">
@@ -18787,12 +18837,12 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>BaP (Brand as Performance)</t>
+          <t>MCB (Marketing Capabilities Benchmark)</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -18802,7 +18852,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>A research study that quantifies the direct impact of branding on business performance and customer acquisition.</t>
+          <t>An assessment system that measures individual team members’ marketing capabilities.</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -18817,12 +18867,12 @@
       </c>
       <c r="K318" t="inlineStr">
         <is>
-          <t>Marka Performansı Araştırması</t>
+          <t>Pazarlama Yetkinlik Kıyaslaması</t>
         </is>
       </c>
       <c r="L318" t="inlineStr">
         <is>
-          <t>Marka algısının satış ve müşteri sadakati üzerindeki etkisini analiz eden çalışma.</t>
+          <t>Pazarlama ekiplerinin yetkinlik düzeylerini belirlemek için kullanılan analiz metodu.</t>
         </is>
       </c>
       <c r="N318" t="inlineStr">
@@ -18834,7 +18884,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>MMGF (Movable Middles Growth Framework)</t>
+          <t>MATT (Marketing Attribution Think Tank)</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -18849,7 +18899,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>A targeting framework that focuses marketing investments on consumer segments most likely to respond to advertising.</t>
+          <t>A think tank dedicated to improving marketing attribution and proving marketing’s impact on business growth.</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
@@ -18864,12 +18914,12 @@
       </c>
       <c r="K319" t="inlineStr">
         <is>
-          <t>Hareketli Ortalar Büyüme Çerçevesi</t>
+          <t>Pazarlama Atıf Düşünce Grubu</t>
         </is>
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t>Pazarlama bütçesini en etkili segmentlere yönlendirmek için kullanılan model.</t>
+          <t>Pazarlama yatırım getirisi (ROI) ve pazarlama performansı ölçümleme konularında çalışan düşünce grubudur.</t>
         </is>
       </c>
       <c r="N319" t="inlineStr">
@@ -18881,12 +18931,12 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>FSS (First Second Strategy)</t>
+          <t>BaP (Brand as Performance)</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -18896,7 +18946,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>A neuroscience-based study analyzing how consumers react to advertising within the first second of exposure.</t>
+          <t>A research study that quantifies the direct impact of branding on business performance and customer acquisition.</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -18911,12 +18961,12 @@
       </c>
       <c r="K320" t="inlineStr">
         <is>
-          <t>İlk Saniye Stratejisi</t>
+          <t>Marka Performansı Araştırması</t>
         </is>
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>Reklamların ilk saniyelerde beyin üzerindeki etkisini inceleyen nöropazarlama araştırması.</t>
+          <t>Marka algısının satış ve müşteri sadakati üzerindeki etkisini analiz eden çalışma.</t>
         </is>
       </c>
       <c r="N320" t="inlineStr">
@@ -18928,12 +18978,12 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>SMoX (Smart Marketing Cross-Effectiveness)</t>
+          <t>MMGF (Movable Middles Growth Framework)</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -18943,7 +18993,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>A research initiative that measures the effectiveness of advertising across multiple media channels.</t>
+          <t>A targeting framework that focuses marketing investments on consumer segments most likely to respond to advertising.</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -18958,12 +19008,12 @@
       </c>
       <c r="K321" t="inlineStr">
         <is>
-          <t>Akıllı Pazarlama Çapraz Etkinlik Araştırmaları</t>
+          <t>Hareketli Ortalar Büyüme Çerçevesi</t>
         </is>
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>Farklı medya kanallarında reklam harcamalarının verimliliğini test eden çalışma.</t>
+          <t>Pazarlama bütçesini en etkili segmentlere yönlendirmek için kullanılan model.</t>
         </is>
       </c>
       <c r="N321" t="inlineStr">
@@ -18975,12 +19025,12 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Project ROMI (Return on Marketing Investment)</t>
+          <t>FSS (First Second Strategy)</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -18990,7 +19040,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>A study connecting marketing investments to financial growth by demonstrating measurable returns.</t>
+          <t>A neuroscience-based study analyzing how consumers react to advertising within the first second of exposure.</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -19005,12 +19055,12 @@
       </c>
       <c r="K322" t="inlineStr">
         <is>
-          <t>Pazarlama Yatırım Getirisi</t>
+          <t>İlk Saniye Stratejisi</t>
         </is>
       </c>
       <c r="L322" t="inlineStr">
         <is>
-          <t>Pazarlamanın işletme büyümesine nasıl katkıda bulunduğunu analiz eden girişim.</t>
+          <t>Reklamların ilk saniyelerde beyin üzerindeki etkisini inceleyen nöropazarlama araştırması.</t>
         </is>
       </c>
       <c r="N322" t="inlineStr">
@@ -19022,12 +19072,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>DATT (Data in Marketing Think Tank)</t>
+          <t>SMoX (Smart Marketing Cross-Effectiveness)</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -19037,7 +19087,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>A think tank dedicated to using data and AI to improve customer experiences and marketing efficiency.</t>
+          <t>A research initiative that measures the effectiveness of advertising across multiple media channels.</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -19052,12 +19102,12 @@
       </c>
       <c r="K323" t="inlineStr">
         <is>
-          <t>Pazarlamada Veri Düşünce Grubu</t>
+          <t>Akıllı Pazarlama Çapraz Etkinlik Araştırmaları</t>
         </is>
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>Veri odaklı pazarlama stratejilerini geliştiren düşünce grubudur.</t>
+          <t>Farklı medya kanallarında reklam harcamalarının verimliliğini test eden çalışma.</t>
         </is>
       </c>
       <c r="N323" t="inlineStr">
@@ -19069,12 +19119,12 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>ROEX (Return on Omnichannel Experience)</t>
+          <t>Project ROMI (Return on Marketing Investment)</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>P</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -19084,7 +19134,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>A study measuring the financial impact of omnichannel customer experiences.</t>
+          <t>A study connecting marketing investments to financial growth by demonstrating measurable returns.</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -19099,12 +19149,12 @@
       </c>
       <c r="K324" t="inlineStr">
         <is>
-          <t>Çok Kanallı Deneyim Getirisi</t>
+          <t>Pazarlama Yatırım Getirisi</t>
         </is>
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>Omnichannel stratejilerin pazarlama getirisi üzerindeki etkisini ölçer.</t>
+          <t>Pazarlamanın işletme büyümesine nasıl katkıda bulunduğunu analiz eden girişim.</t>
         </is>
       </c>
       <c r="N324" t="inlineStr">
@@ -19116,12 +19166,12 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>CAP (Consortium for AI Personalization)</t>
+          <t>DATT (Data in Marketing Think Tank)</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -19131,7 +19181,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>A collaborative initiative exploring the role of AI in personalizing marketing and customer interactions.</t>
+          <t>A think tank dedicated to using data and AI to improve customer experiences and marketing efficiency.</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
@@ -19146,12 +19196,12 @@
       </c>
       <c r="K325" t="inlineStr">
         <is>
-          <t>Yapay Zeka Kişiselleştirme Konsorsiyumu</t>
+          <t>Pazarlamada Veri Düşünce Grubu</t>
         </is>
       </c>
       <c r="L325" t="inlineStr">
         <is>
-          <t>Yapay zeka ile kişiselleştirilmiş pazarlama stratejileri geliştiren bir konsorsiyum.</t>
+          <t>Veri odaklı pazarlama stratejilerini geliştiren düşünce grubudur.</t>
         </is>
       </c>
       <c r="N325" t="inlineStr">
@@ -19163,12 +19213,12 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>ALC (AI Leadership Coalition)</t>
+          <t>ROEX (Return on Omnichannel Experience)</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -19178,7 +19228,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>A think tank focused on advancing the responsible use of AI in marketing.</t>
+          <t>A study measuring the financial impact of omnichannel customer experiences.</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
@@ -19193,12 +19243,12 @@
       </c>
       <c r="K326" t="inlineStr">
         <is>
-          <t>Yapay Zeka Liderlik Koalisyonu</t>
+          <t>Çok Kanallı Deneyim Getirisi</t>
         </is>
       </c>
       <c r="L326" t="inlineStr">
         <is>
-          <t>Yapay zeka (AI) kullanımını pazarlamada optimize eden girişimdir.</t>
+          <t>Omnichannel stratejilerin pazarlama getirisi üzerindeki etkisini ölçer.</t>
         </is>
       </c>
       <c r="N326" t="inlineStr">
@@ -19210,12 +19260,12 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>RAIL (Responsible AI Innovation Lab)</t>
+          <t>CAP (Consortium for AI Personalization)</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -19225,7 +19275,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>A research group developing ethical and practical AI applications for marketing.</t>
+          <t>A collaborative initiative exploring the role of AI in personalizing marketing and customer interactions.</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -19240,12 +19290,12 @@
       </c>
       <c r="K327" t="inlineStr">
         <is>
-          <t>Sorumlu Yapay Zeka İnovasyon Laboratuvarı</t>
+          <t>Yapay Zeka Kişiselleştirme Konsorsiyumu</t>
         </is>
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t>Pazarlamada yapay zekanın etik ve güvenilir kullanımı üzerine çalışmalar yürütür.</t>
+          <t>Yapay zeka ile kişiselleştirilmiş pazarlama stratejileri geliştiren bir konsorsiyum.</t>
         </is>
       </c>
       <c r="N327" t="inlineStr">
@@ -19257,12 +19307,12 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>SAVE (Brand Safety Council Initiative)</t>
+          <t>ALC (AI Leadership Coalition)</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -19272,7 +19322,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>An initiative to develop brand-safe advertising practices and reduce digital advertising risks.</t>
+          <t>A think tank focused on advancing the responsible use of AI in marketing.</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -19287,12 +19337,12 @@
       </c>
       <c r="K328" t="inlineStr">
         <is>
-          <t>Marka Güvenliği Konseyi Girişimi</t>
+          <t>Yapay Zeka Liderlik Koalisyonu</t>
         </is>
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>Markaların güvenli reklam stratejileri oluşturmasını sağlayan girişim.</t>
+          <t>Yapay zeka (AI) kullanımını pazarlamada optimize eden girişimdir.</t>
         </is>
       </c>
       <c r="N328" t="inlineStr">
@@ -19304,12 +19354,12 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SMARTIES (Business Impact Awards)</t>
+          <t>RAIL (Responsible AI Innovation Lab)</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -19319,7 +19369,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>A global award program recognizing marketing innovation and business impact in mobile and digital marketing.</t>
+          <t>A research group developing ethical and practical AI applications for marketing.</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -19334,12 +19384,12 @@
       </c>
       <c r="K329" t="inlineStr">
         <is>
-          <t>İş Etkisi Ödülleri</t>
+          <t>Sorumlu Yapay Zeka İnovasyon Laboratuvarı</t>
         </is>
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t>Mobil pazarlamada yenilikçi stratejiler geliştiren markalara verilen ödüller.</t>
+          <t>Pazarlamada yapay zekanın etik ve güvenilir kullanımı üzerine çalışmalar yürütür.</t>
         </is>
       </c>
       <c r="N329" t="inlineStr">
@@ -19351,12 +19401,12 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>BII (Business Impact Index)</t>
+          <t>SAVE (Brand Safety Council Initiative)</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -19366,7 +19416,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>An index that evaluates the business performance of SMARTIES award-winning campaigns.</t>
+          <t>An initiative to develop brand-safe advertising practices and reduce digital advertising risks.</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -19381,12 +19431,12 @@
       </c>
       <c r="K330" t="inlineStr">
         <is>
-          <t>SMARTIES İş Etki Endeksi</t>
+          <t>Marka Güvenliği Konseyi Girişimi</t>
         </is>
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t>SMARTIES ödüllerinin iş etkisini analiz eden endeks.</t>
+          <t>Markaların güvenli reklam stratejileri oluşturmasını sağlayan girişim.</t>
         </is>
       </c>
       <c r="N330" t="inlineStr">
@@ -19398,12 +19448,12 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>MM25 (Peer Group for Marketing Executives)</t>
+          <t>SMARTIES (Business Impact Awards)</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -19413,7 +19463,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>A networking and knowledge-sharing group for senior marketing leaders.</t>
+          <t>A global award program recognizing marketing innovation and business impact in mobile and digital marketing.</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -19428,12 +19478,12 @@
       </c>
       <c r="K331" t="inlineStr">
         <is>
-          <t>Pazarlama Yöneticileri İçin Meslektaş Grubu</t>
+          <t>İş Etkisi Ödülleri</t>
         </is>
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t>Pazarlama liderleri için oluşturulmuş bir bilgi paylaşım platformu.</t>
+          <t>Mobil pazarlamada yenilikçi stratejiler geliştiren markalara verilen ödüller.</t>
         </is>
       </c>
       <c r="N331" t="inlineStr">
@@ -19445,12 +19495,12 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>MAdopt (Marketer Adoption Initiative)</t>
+          <t>BII (Business Impact Index)</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -19460,7 +19510,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>An initiative to increase the adoption of MMA’s marketing tools and best practices among members.</t>
+          <t>An index that evaluates the business performance of SMARTIES award-winning campaigns.</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
@@ -19475,12 +19525,12 @@
       </c>
       <c r="K332" t="inlineStr">
         <is>
-          <t>Pazarlama Benimseme Girişimi</t>
+          <t>SMARTIES İş Etki Endeksi</t>
         </is>
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>MMA’nin sunduğu araçların pazarlamacılar tarafından benimsenmesini teşvik eden girişim.</t>
+          <t>SMARTIES ödüllerinin iş etkisini analiz eden endeks.</t>
         </is>
       </c>
       <c r="N332" t="inlineStr">
@@ -19492,12 +19542,12 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>SMO (Social Media Optimization)</t>
+          <t>MM25 (Peer Group for Marketing Executives)</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -19507,7 +19557,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Techniques to enhance visibility and interaction on social media.</t>
+          <t>A networking and knowledge-sharing group for senior marketing leaders.</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -19517,12 +19567,17 @@
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>Digital Marketing Acronyms</t>
+          <t>MMA Programs &amp; Frameworks</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Pazarlama Yöneticileri İçin Meslektaş Grubu</t>
         </is>
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t>Sosyal medya içeriklerinin görünürlüğünü artırma teknikleri.</t>
+          <t>Pazarlama liderleri için oluşturulmuş bir bilgi paylaşım platformu.</t>
         </is>
       </c>
       <c r="N333" t="inlineStr">
@@ -19534,12 +19589,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>UGC (User-Generated Content)</t>
+          <t>MAdopt (Marketer Adoption Initiative)</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -19549,7 +19604,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Content created by users (comments, posts, videos).</t>
+          <t>An initiative to increase the adoption of MMA’s marketing tools and best practices among members.</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
@@ -19559,12 +19614,17 @@
       </c>
       <c r="J334" t="inlineStr">
         <is>
-          <t>Digital Marketing Acronyms</t>
+          <t>MMA Programs &amp; Frameworks</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Pazarlama Benimseme Girişimi</t>
         </is>
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t>Kullanıcılar tarafından oluşturulan içerik.</t>
+          <t>MMA’nin sunduğu araçların pazarlamacılar tarafından benimsenmesini teşvik eden girişim.</t>
         </is>
       </c>
       <c r="N334" t="inlineStr">
@@ -19576,12 +19636,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>TAT (Turnaround Time)</t>
+          <t>SMO (Social Media Optimization)</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -19591,7 +19651,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Response time to customer queries.</t>
+          <t>Techniques to enhance visibility and interaction on social media.</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -19606,7 +19666,7 @@
       </c>
       <c r="L335" t="inlineStr">
         <is>
-          <t>Müşteri sorularına cevap verme süresi.</t>
+          <t>Sosyal medya içeriklerinin görünürlüğünü artırma teknikleri.</t>
         </is>
       </c>
       <c r="N335" t="inlineStr">
@@ -19618,12 +19678,12 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>CTR (Content Traffic Rate)</t>
+          <t>UGC (User-Generated Content)</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>U</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -19633,7 +19693,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Measures the traffic driven by social media content to websites or landing pages.</t>
+          <t>Content created by users (comments, posts, videos).</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -19648,29 +19708,24 @@
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>İçeriğin web sitesine yönlendirdiği trafik oranı.</t>
+          <t>Kullanıcılar tarafından oluşturulan içerik.</t>
         </is>
       </c>
       <c r="N336" t="inlineStr">
         <is>
           <t>Source list</t>
-        </is>
-      </c>
-      <c r="Q336" t="inlineStr">
-        <is>
-          <t>Source list expands CTR as 'Content Traffic Rate', which is non-standard; CTR usually means Click-Through Rate (see that entry).</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>ENG% (Engagement Rate)</t>
+          <t>TAT (Turnaround Time)</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -19680,7 +19735,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Measures post likes, comments, shares, and saves.</t>
+          <t>Response time to customer queries.</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -19695,7 +19750,7 @@
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>Gönderilerin beğeni, yorum, paylaşım oranı.</t>
+          <t>Müşteri sorularına cevap verme süresi.</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
@@ -19707,12 +19762,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>ORM (Online Reputation Management)</t>
+          <t>CTR (Content Traffic Rate)</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -19722,7 +19777,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Process of managing a brand's online reputation.</t>
+          <t>Measures the traffic driven by social media content to websites or landing pages.</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -19737,24 +19792,29 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>Online itibar yönetimi.</t>
+          <t>İçeriğin web sitesine yönlendirdiği trafik oranı.</t>
         </is>
       </c>
       <c r="N338" t="inlineStr">
         <is>
           <t>Source list</t>
+        </is>
+      </c>
+      <c r="Q338" t="inlineStr">
+        <is>
+          <t>Source list expands CTR as 'Content Traffic Rate', which is non-standard; CTR usually means Click-Through Rate (see that entry).</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>KOC (Key Opinion Consumer)</t>
+          <t>ENG% (Engagement Rate)</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -19764,7 +19824,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Influential individuals whose opinions affect consumer decisions.</t>
+          <t>Measures post likes, comments, shares, and saves.</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -19779,7 +19839,7 @@
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t>Tüketiciyi etkileyen mikro influencer.</t>
+          <t>Gönderilerin beğeni, yorum, paylaşım oranı.</t>
         </is>
       </c>
       <c r="N339" t="inlineStr">
@@ -19791,12 +19851,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>EPM (Engagement Per Mille)</t>
+          <t>ORM (Online Reputation Management)</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>O</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -19806,7 +19866,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Interaction rate per 1,000 impressions.</t>
+          <t>Process of managing a brand's online reputation.</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -19821,7 +19881,7 @@
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t>1000 gösterim başına etkileşim.</t>
+          <t>Online itibar yönetimi.</t>
         </is>
       </c>
       <c r="N340" t="inlineStr">
@@ -19833,12 +19893,12 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>A/B Testing (Split Testing)</t>
+          <t>KOC (Key Opinion Consumer)</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -19848,7 +19908,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Comparing two versions of content to determine the most effective one.</t>
+          <t>Influential individuals whose opinions affect consumer decisions.</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -19863,7 +19923,7 @@
       </c>
       <c r="L341" t="inlineStr">
         <is>
-          <t>İki içerik arasında karşılaştırma yaparak en iyisini seçme.</t>
+          <t>Tüketiciyi etkileyen mikro influencer.</t>
         </is>
       </c>
       <c r="N341" t="inlineStr">
@@ -19875,12 +19935,12 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>LTV (Customer Lifetime Value)</t>
+          <t>EPM (Engagement Per Mille)</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -19890,7 +19950,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Total revenue value of a customer to a brand.</t>
+          <t>Interaction rate per 1,000 impressions.</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -19905,7 +19965,7 @@
       </c>
       <c r="L342" t="inlineStr">
         <is>
-          <t>Müşterinin marka için toplam gelir değeri.</t>
+          <t>1000 gösterim başına etkileşim.</t>
         </is>
       </c>
       <c r="N342" t="inlineStr">
@@ -19917,12 +19977,12 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CR (Conversion Rate)</t>
+          <t>A/B Testing (Split Testing)</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -19932,7 +19992,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Rate of conversion from ads or campaigns.</t>
+          <t>Comparing two versions of content to determine the most effective one.</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -19947,7 +20007,7 @@
       </c>
       <c r="L343" t="inlineStr">
         <is>
-          <t>Dönüşüm oranı.</t>
+          <t>İki içerik arasında karşılaştırma yaparak en iyisini seçme.</t>
         </is>
       </c>
       <c r="N343" t="inlineStr">
@@ -19959,12 +20019,12 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>CPL (Cost Per Lead)</t>
+          <t>LTV (Customer Lifetime Value)</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -19974,7 +20034,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Cost of acquiring a new lead.</t>
+          <t>Total revenue value of a customer to a brand.</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -19989,7 +20049,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t>Potansiyel müşteri kazanma maliyeti.</t>
+          <t>Müşterinin marka için toplam gelir değeri.</t>
         </is>
       </c>
       <c r="N344" t="inlineStr">
@@ -20001,7 +20061,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>CPV (Cost Per View)</t>
+          <t>CR (Conversion Rate)</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -20016,7 +20076,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Cost paid per view in video ads.</t>
+          <t>Rate of conversion from ads or campaigns.</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -20031,7 +20091,7 @@
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t>Görüntüleme başına maliyet.</t>
+          <t>Dönüşüm oranı.</t>
         </is>
       </c>
       <c r="N345" t="inlineStr">
@@ -20043,12 +20103,12 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>VTR (View-Through Rate)</t>
+          <t>CPL (Cost Per Lead)</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -20058,7 +20118,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>Users who convert later after viewing ads without immediate clicking.</t>
+          <t>Cost of acquiring a new lead.</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -20073,29 +20133,24 @@
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t>Reklam sonrası gecikmeli dönüşüm oranı.</t>
+          <t>Potansiyel müşteri kazanma maliyeti.</t>
         </is>
       </c>
       <c r="N346" t="inlineStr">
         <is>
           <t>Source list</t>
-        </is>
-      </c>
-      <c r="Q346" t="inlineStr">
-        <is>
-          <t>Source definition describes view-through conversion; VTR usually means the share of viewers who watch a video ad to completion. Check before publishing.</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>DSP (Demand-Side Platform)</t>
+          <t>CPV (Cost Per View)</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -20105,7 +20160,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>Platform for buying digital ad inventory.</t>
+          <t>Cost paid per view in video ads.</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -20120,7 +20175,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t>Reklamverenlerin dijital reklam alanını otomatik olarak satın aldığı platformdur.</t>
+          <t>Görüntüleme başına maliyet.</t>
         </is>
       </c>
       <c r="N347" t="inlineStr">
@@ -20132,12 +20187,12 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>SSP (Supply-Side Platform)</t>
+          <t>VTR (View-Through Rate)</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>V</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -20147,7 +20202,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Platform for publishers to manage and sell ad inventory.</t>
+          <t>Users who convert later after viewing ads without immediate clicking.</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -20162,24 +20217,29 @@
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t>Yayıncıların reklam envanterini yönetip otomatik olarak sattığı platformdur.</t>
+          <t>Reklam sonrası gecikmeli dönüşüm oranı.</t>
         </is>
       </c>
       <c r="N348" t="inlineStr">
         <is>
           <t>Source list</t>
+        </is>
+      </c>
+      <c r="Q348" t="inlineStr">
+        <is>
+          <t>Source definition describes view-through conversion; VTR usually means the share of viewers who watch a video ad to completion. Check before publishing.</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>SEM (Search Engine Marketing)</t>
+          <t>DSP (Demand-Side Platform)</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -20189,7 +20249,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>Advertising through paid search results.</t>
+          <t>Platform for buying digital ad inventory.</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -20204,7 +20264,7 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t>Arama motorlarındaki ücretli sonuçlar aracılığıyla yapılan reklamcılıktır.</t>
+          <t>Reklamverenlerin dijital reklam alanını otomatik olarak satın aldığı platformdur.</t>
         </is>
       </c>
       <c r="N349" t="inlineStr">
@@ -20216,7 +20276,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>SERP (Search Engine Results Page)</t>
+          <t>SSP (Supply-Side Platform)</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -20231,7 +20291,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Page shown by a search engine in response to a query.</t>
+          <t>Platform for publishers to manage and sell ad inventory.</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -20246,7 +20306,7 @@
       </c>
       <c r="L350" t="inlineStr">
         <is>
-          <t>Arama motoru sonuç sayfası.</t>
+          <t>Yayıncıların reklam envanterini yönetip otomatik olarak sattığı platformdur.</t>
         </is>
       </c>
       <c r="N350" t="inlineStr">
@@ -20258,12 +20318,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>DA (Domain Authority)</t>
+          <t>SEM (Search Engine Marketing)</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -20273,7 +20333,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Score indicating website strength in search engines.</t>
+          <t>Advertising through paid search results.</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -20288,7 +20348,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t>Web sitesinin gücünü gösteren skor.</t>
+          <t>Arama motorlarındaki ücretli sonuçlar aracılığıyla yapılan reklamcılıktır.</t>
         </is>
       </c>
       <c r="N351" t="inlineStr">
@@ -20300,12 +20360,12 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>BR (Bounce Rate)</t>
+          <t>SERP (Search Engine Results Page)</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -20315,7 +20375,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Rate at which visitors leave the site without interaction.</t>
+          <t>Page shown by a search engine in response to a query.</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -20330,7 +20390,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t>Hemen çıkma oranı.</t>
+          <t>Arama motoru sonuç sayfası.</t>
         </is>
       </c>
       <c r="N352" t="inlineStr">
@@ -20342,12 +20402,12 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>RO (Reach &amp; Overlap)</t>
+          <t>DA (Domain Authority)</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -20357,7 +20417,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>Measures audience overlap across platforms.</t>
+          <t>Score indicating website strength in search engines.</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -20372,7 +20432,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t>Farklı platformlardaki kitlelerin ne kadar örtüştüğünü ölçen metriktir.</t>
+          <t>Web sitesinin gücünü gösteren skor.</t>
         </is>
       </c>
       <c r="N353" t="inlineStr">
@@ -20384,12 +20444,12 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>SEO (Search Engine Optimization)</t>
+          <t>BR (Bounce Rate)</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -20399,7 +20459,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Techniques to improve visibility in organic search results.</t>
+          <t>Rate at which visitors leave the site without interaction.</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
@@ -20414,7 +20474,7 @@
       </c>
       <c r="L354" t="inlineStr">
         <is>
-          <t>Arama motoru optimizasyonu teknikleri.</t>
+          <t>Hemen çıkma oranı.</t>
         </is>
       </c>
       <c r="N354" t="inlineStr">
@@ -20426,12 +20486,12 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>GA (Google Analytics)</t>
+          <t>RO (Reach &amp; Overlap)</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -20441,7 +20501,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>Web analytics service by Google.</t>
+          <t>Measures audience overlap across platforms.</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -20456,7 +20516,7 @@
       </c>
       <c r="L355" t="inlineStr">
         <is>
-          <t>Google web analizi hizmeti.</t>
+          <t>Farklı platformlardaki kitlelerin ne kadar örtüştüğünü ölçen metriktir.</t>
         </is>
       </c>
       <c r="N355" t="inlineStr">
@@ -20468,12 +20528,12 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>UX (User Experience)</t>
+          <t>SEO (Search Engine Optimization)</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -20483,7 +20543,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>Overall experience of a user with a product or service.</t>
+          <t>Techniques to improve visibility in organic search results.</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -20498,7 +20558,7 @@
       </c>
       <c r="L356" t="inlineStr">
         <is>
-          <t>Kullanıcının bir ürün ya da hizmetle yaşadığı deneyimin bütünüdür.</t>
+          <t>Arama motoru optimizasyonu teknikleri.</t>
         </is>
       </c>
       <c r="N356" t="inlineStr">
@@ -20510,12 +20570,12 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>TOFU (Top of Funnel)</t>
+          <t>GA (Google Analytics)</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -20525,7 +20585,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Content aimed at awareness for new customers.</t>
+          <t>Web analytics service by Google.</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -20540,7 +20600,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t>Huninin üst aşaması (farkındalık).</t>
+          <t>Google web analizi hizmeti.</t>
         </is>
       </c>
       <c r="N357" t="inlineStr">
@@ -20552,12 +20612,12 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>MOFU (Middle of Funnel)</t>
+          <t>UX (User Experience)</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>U</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -20567,7 +20627,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Content aimed at increasing interest of potential customers.</t>
+          <t>Overall experience of a user with a product or service.</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -20582,7 +20642,7 @@
       </c>
       <c r="L358" t="inlineStr">
         <is>
-          <t>Huninin orta aşaması (ilgi).</t>
+          <t>Kullanıcının bir ürün ya da hizmetle yaşadığı deneyimin bütünüdür.</t>
         </is>
       </c>
       <c r="N358" t="inlineStr">
@@ -20594,12 +20654,12 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>BOFU (Bottom of Funnel)</t>
+          <t>TOFU (Top of Funnel)</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>T</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -20609,7 +20669,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Conversion-focused content (offers, discounts, demos).</t>
+          <t>Content aimed at awareness for new customers.</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -20624,7 +20684,7 @@
       </c>
       <c r="L359" t="inlineStr">
         <is>
-          <t>Huninin alt aşaması (dönüşüm).</t>
+          <t>Huninin üst aşaması (farkındalık).</t>
         </is>
       </c>
       <c r="N359" t="inlineStr">
@@ -20636,12 +20696,12 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>CAC (Customer Acquisition Cost)</t>
+          <t>MOFU (Middle of Funnel)</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -20651,7 +20711,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>Cost of gaining a new customer.</t>
+          <t>Content aimed at increasing interest of potential customers.</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -20666,7 +20726,7 @@
       </c>
       <c r="L360" t="inlineStr">
         <is>
-          <t>Müşteri kazanma maliyeti.</t>
+          <t>Huninin orta aşaması (ilgi).</t>
         </is>
       </c>
       <c r="N360" t="inlineStr">
@@ -20678,12 +20738,12 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>MQL (Marketing Qualified Lead)</t>
+          <t>BOFU (Bottom of Funnel)</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -20693,7 +20753,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>A potential customer ready for sales engagement.</t>
+          <t>Conversion-focused content (offers, discounts, demos).</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -20708,7 +20768,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t>Pazarlama faaliyetleri sonucunda satış ekibine aktarılmaya hazır hale gelen potansiyel müşteridir.</t>
+          <t>Huninin alt aşaması (dönüşüm).</t>
         </is>
       </c>
       <c r="N361" t="inlineStr">
@@ -20720,12 +20780,12 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>SQL (Sales Qualified Lead)</t>
+          <t>CAC (Customer Acquisition Cost)</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -20735,7 +20795,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Lead evaluated by sales team ready for direct engagement.</t>
+          <t>Cost of gaining a new customer.</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -20750,7 +20810,7 @@
       </c>
       <c r="L362" t="inlineStr">
         <is>
-          <t>Satış ekibi tarafından değerlendirilmiş ve doğrudan satış görüşmesine hazır potansiyel müşteridir.</t>
+          <t>Müşteri kazanma maliyeti.</t>
         </is>
       </c>
       <c r="N362" t="inlineStr">
@@ -20762,12 +20822,12 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>GA4 (Google Analytics 4)</t>
+          <t>MQL (Marketing Qualified Lead)</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -20777,7 +20837,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>Google’s advanced analytics platform for tracking user interactions.</t>
+          <t>A potential customer ready for sales engagement.</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -20792,7 +20852,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t>Google'ın web sitesi ve uygulamalardaki kullanıcı etkileşimlerini birlikte ölçen analitik platformudur.</t>
+          <t>Pazarlama faaliyetleri sonucunda satış ekibine aktarılmaya hazır hale gelen potansiyel müşteridir.</t>
         </is>
       </c>
       <c r="N363" t="inlineStr">
@@ -20804,12 +20864,12 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>BI (Business Intelligence)</t>
+          <t>SQL (Sales Qualified Lead)</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -20819,7 +20879,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Systems analyzing business data for better decisions.</t>
+          <t>Lead evaluated by sales team ready for direct engagement.</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -20834,7 +20894,7 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>Şirket verisini analiz ederek daha iyi karar almayı sağlayan sistemlerdir.</t>
+          <t>Satış ekibi tarafından değerlendirilmiş ve doğrudan satış görüşmesine hazır potansiyel müşteridir.</t>
         </is>
       </c>
       <c r="N364" t="inlineStr">
@@ -20846,12 +20906,12 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>DTC (Direct-to-Consumer)</t>
+          <t>GA4 (Google Analytics 4)</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -20861,7 +20921,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Business model selling directly to consumers without intermediaries.</t>
+          <t>Google’s advanced analytics platform for tracking user interactions.</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -20876,7 +20936,7 @@
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>Markanın aracı kullanmadan doğrudan tüketiciye sattığı iş modelidir.</t>
+          <t>Google'ın web sitesi ve uygulamalardaki kullanıcı etkileşimlerini birlikte ölçen analitik platformudur.</t>
         </is>
       </c>
       <c r="N365" t="inlineStr">
@@ -20888,12 +20948,12 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>UGR (User-Generated Reviews)</t>
+          <t>BI (Business Intelligence)</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -20903,7 +20963,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Reviews created by users that build trust in brands.</t>
+          <t>Systems analyzing business data for better decisions.</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -20918,7 +20978,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>Kullanıcıların yazdığı, markaya güven oluşturan değerlendirmelerdir.</t>
+          <t>Şirket verisini analiz ederek daha iyi karar almayı sağlayan sistemlerdir.</t>
         </is>
       </c>
       <c r="N366" t="inlineStr">
@@ -20930,12 +20990,12 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>CX (Customer Experience)</t>
+          <t>DTC (Direct-to-Consumer)</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -20945,7 +21005,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>Overall interaction experience between customer and brand.</t>
+          <t>Business model selling directly to consumers without intermediaries.</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -20960,7 +21020,7 @@
       </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t>Müşterinin markayla tüm temas noktalarında yaşadığı deneyimin bütünüdür.</t>
+          <t>Markanın aracı kullanmadan doğrudan tüketiciye sattığı iş modelidir.</t>
         </is>
       </c>
       <c r="N367" t="inlineStr">
@@ -20972,12 +21032,12 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>RTM (Real-Time Marketing)</t>
+          <t>UGR (User-Generated Reviews)</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>U</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20987,7 +21047,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Instant marketing responding to current events.</t>
+          <t>Reviews created by users that build trust in brands.</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -21002,7 +21062,7 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t>Güncel olaylara ve anlık gelişmelere hızla yanıt veren pazarlamadır.</t>
+          <t>Kullanıcıların yazdığı, markaya güven oluşturan değerlendirmelerdir.</t>
         </is>
       </c>
       <c r="N368" t="inlineStr">
@@ -21014,12 +21074,12 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>UGS (User-Generated Stories)</t>
+          <t>CX (Customer Experience)</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -21029,7 +21089,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Stories created by users enhancing brand authenticity.</t>
+          <t>Overall interaction experience between customer and brand.</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -21044,7 +21104,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t>Kullanıcıların oluşturduğu, markanın samimiyetini güçlendiren hikayelerdir.</t>
+          <t>Müşterinin markayla tüm temas noktalarında yaşadığı deneyimin bütünüdür.</t>
         </is>
       </c>
       <c r="N369" t="inlineStr">
@@ -21056,40 +21116,124 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
+          <t>RTM (Real-Time Marketing)</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>EN/TR</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Instant marketing responding to current events.</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>MMA Sözlük / MMA Acronyms.docx</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>Digital Marketing Acronyms</t>
+        </is>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>Güncel olaylara ve anlık gelişmelere hızla yanıt veren pazarlamadır.</t>
+        </is>
+      </c>
+      <c r="N370" t="inlineStr">
+        <is>
+          <t>Source list</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>UGS (User-Generated Stories)</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>EN/TR</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Stories created by users enhancing brand authenticity.</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>MMA Sözlük / MMA Acronyms.docx</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>Digital Marketing Acronyms</t>
+        </is>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>Kullanıcıların oluşturduğu, markanın samimiyetini güçlendiren hikayelerdir.</t>
+        </is>
+      </c>
+      <c r="N371" t="inlineStr">
+        <is>
+          <t>Source list</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
           <t>CTA (Call to Action)</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
+      <c r="B372" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t>EN/TR</t>
-        </is>
-      </c>
-      <c r="D370" t="inlineStr">
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>EN/TR</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
         <is>
           <t>Calls directing users to specific actions (e.g., "Buy Now", "Register").</t>
         </is>
       </c>
-      <c r="G370" t="inlineStr">
+      <c r="G372" t="inlineStr">
         <is>
           <t>MMA Sözlük / MMA Acronyms.docx</t>
         </is>
       </c>
-      <c r="J370" t="inlineStr">
+      <c r="J372" t="inlineStr">
         <is>
           <t>Digital Marketing Acronyms</t>
         </is>
       </c>
-      <c r="L370" t="inlineStr">
+      <c r="L372" t="inlineStr">
         <is>
           <t>Kullanıcıyı belirli bir eyleme yönlendiren ifadedir; "Şimdi Satın Al" ya da "Kaydol" gibi.</t>
         </is>
       </c>
-      <c r="N370" t="inlineStr">
+      <c r="N372" t="inlineStr">
         <is>
           <t>Source list</t>
         </is>

</xml_diff>